<commit_message>
Fix Cloudflare Pages build v3.3.20
</commit_message>
<xml_diff>
--- a/templates/SubsTracker_账号数据库批量导入模板.xlsx
+++ b/templates/SubsTracker_账号数据库批量导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账号导入" sheetId="1" r:id="R6764f23f5a63494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R223b319246b0487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账号导入" sheetId="1" r:id="Rbf91cf23765f4223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R04b66afbb72b426a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -33,8 +33,13 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -51,6 +56,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -59,7 +69,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="24">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -100,6 +110,10 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -310,6 +324,7 @@
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -337,10 +352,13 @@
       <x:c r="H1" s="10" t="str">
         <x:v>QQ密码</x:v>
       </x:c>
+      <x:c r="I1" s="23" t="str">
+        <x:v>公/私</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="14" t="str">
-        <x:v>001</x:v>
+        <x:v>公司01号</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
         <x:v>user@example.com</x:v>
@@ -363,10 +381,13 @@
       <x:c r="H2" s="14" t="str">
         <x:v>QQPass</x:v>
       </x:c>
+      <x:c r="I2" t="str">
+        <x:v>公司</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="14" t="str">
-        <x:v>002</x:v>
+        <x:v>个人01号</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
         <x:v>13800138000</x:v>
@@ -381,6 +402,9 @@
       <x:c r="F3" s="14" t="str"/>
       <x:c r="G3" s="14" t="str"/>
       <x:c r="H3" s="14" t="str"/>
+      <x:c r="I3" t="str">
+        <x:v>个人</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="14" t="str">
@@ -399,6 +423,9 @@
       <x:c r="F4" s="14" t="str"/>
       <x:c r="G4" s="14" t="str"/>
       <x:c r="H4" s="14" t="str"/>
+      <x:c r="I4" t="str">
+        <x:v>公司</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="14" t="str">
@@ -417,6 +444,9 @@
       <x:c r="F5" s="14" t="str"/>
       <x:c r="G5" s="14" t="str"/>
       <x:c r="H5" s="14" t="str"/>
+      <x:c r="I5" t="str">
+        <x:v>公司</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="14"/>
@@ -10369,6 +10399,11 @@
       <x:c r="H1000" s="14"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I500">
+      <x:formula1>"公司,个人"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -10447,7 +10482,7 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>自由文本，例如：手机号、邮箱、微信、QQ、平台账号、配音供应商。</x:v>
+        <x:v>基础资料库提供账号类型菜单。导入自定义类型后也会出现在新增账号菜单中。</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
         <x:v>已有账号导入非空值时更新；留空保留原值。</x:v>
@@ -10541,6 +10576,20 @@
       <x:c r="C14" s="11" t="str"/>
       <x:c r="D14" s="11" t="str"/>
     </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>公/私</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>仅可填写“公司”或“个人”。新增账号窗口根据此选项自动编号；Excel导入仍保留所填账号序号。</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>留空时由公司/个人序号前缀识别，否则保留已有资料，不猜测归属。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A11:D11"/>

</xml_diff>